<commit_message>
UI: Improve DemoAppSection card styling and mobile spacing. FIX: Enhance Excel download cache-busting logic.
</commit_message>
<xml_diff>
--- a/public/skillsheet.xlsx
+++ b/public/skillsheet.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F47646D0-3900-4D4E-A614-91A4A2D2D0DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CDA6F60-0279-426F-AA03-3FAC411A15A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1670" yWindow="30" windowWidth="24200" windowHeight="20850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="スキルシート" sheetId="1" r:id="rId1"/>
@@ -303,13 +303,6 @@
     <t>https://melody-muse-neon.vercel.app/</t>
   </si>
   <si>
-    <t>作成日: 2026年4月2日</t>
-    <rPh sb="0" eb="2">
-      <t>サクセイ</t>
-    </rPh>
-    <phoneticPr fontId="12"/>
-  </si>
-  <si>
     <t>★★★★☆</t>
     <phoneticPr fontId="12"/>
   </si>
@@ -469,35 +462,37 @@
     <phoneticPr fontId="12"/>
   </si>
   <si>
-    <t>Figma
-Outlook
-Teams
-Backlog
-UI/UX設計
-UXリサーチ
-ユーザビリティテスト
-プロトタイプ作成
-デザインシステム構築</t>
+    <t>■  主な制作実績（AIを活用した個人開発）</t>
+    <rPh sb="13" eb="15">
+      <t>カツヨウ</t>
+    </rPh>
+    <phoneticPr fontId="12"/>
+  </si>
+  <si>
+    <t>使用言語など</t>
+    <rPh sb="2" eb="4">
+      <t>ゲンゴ</t>
+    </rPh>
+    <phoneticPr fontId="12"/>
+  </si>
+  <si>
+    <t>HTML / CSS</t>
     <phoneticPr fontId="12"/>
   </si>
   <si>
     <t>Figma
 Teams
 Slack
-UI/UX設計
-デザインシステム
-プロトタイプ作成
+競合調査
+課題再定義
+ユーザービリティレビュー
 レスポンシブ</t>
-    <phoneticPr fontId="12"/>
-  </si>
-  <si>
-    <t>Figma
-Notion
-VS Code
-Slack
-Quasar
-Vue.js
-UI設計</t>
+    <rPh sb="19" eb="23">
+      <t>キョウゴウチョウサ</t>
+    </rPh>
+    <rPh sb="24" eb="29">
+      <t>カダイサイテイギ</t>
+    </rPh>
     <phoneticPr fontId="12"/>
   </si>
   <si>
@@ -517,21 +512,43 @@
     <phoneticPr fontId="12"/>
   </si>
   <si>
-    <t>■  主な制作実績（AIを活用した個人開発）</t>
-    <rPh sb="13" eb="15">
-      <t>カツヨウ</t>
-    </rPh>
-    <phoneticPr fontId="12"/>
-  </si>
-  <si>
-    <t>使用言語など</t>
-    <rPh sb="2" eb="4">
-      <t>ゲンゴ</t>
-    </rPh>
-    <phoneticPr fontId="12"/>
-  </si>
-  <si>
-    <t>HTML / CSS</t>
+    <t>Figma
+Notion
+VS Code
+Slack
+Quasar（Vue.js）
+競合調査
+UXリサーチ
+ユーザビリティテスト</t>
+    <phoneticPr fontId="12"/>
+  </si>
+  <si>
+    <t>Figma
+Outlook
+Teams
+Backlog
+競合調査
+UXリサーチ
+ユーザビリティテスト
+ペルソナ作成
+カスタマジャーニーマップ
+ヒューリスティック評価</t>
+    <rPh sb="29" eb="33">
+      <t>キョウゴウチョウサ</t>
+    </rPh>
+    <rPh sb="56" eb="58">
+      <t>サクセイ</t>
+    </rPh>
+    <rPh sb="81" eb="83">
+      <t>ヒョウカ</t>
+    </rPh>
+    <phoneticPr fontId="12"/>
+  </si>
+  <si>
+    <t>作成日: 2026年4月14日</t>
+    <rPh sb="0" eb="2">
+      <t>サクセイ</t>
+    </rPh>
     <phoneticPr fontId="12"/>
   </si>
 </sst>
@@ -539,7 +556,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -640,6 +657,14 @@
       <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="9">
@@ -743,7 +768,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -775,6 +800,41 @@
     <xf numFmtId="0" fontId="13" fillId="8" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
@@ -784,47 +844,15 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
@@ -1174,149 +1202,149 @@
     <col min="1" max="1" width="14.7265625" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="22" customWidth="1"/>
+    <col min="7" max="7" width="23.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
     </row>
     <row r="2" spans="1:7" ht="2.65" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="28"/>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
+      <c r="A2" s="12"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
     </row>
     <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.4">
-      <c r="A3" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
+      <c r="A3" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
     </row>
     <row r="4" spans="1:7" ht="14.65" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
     </row>
     <row r="5" spans="1:7" ht="13.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="26" t="s">
+      <c r="B5" s="14"/>
+      <c r="C5" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" ht="13.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="25"/>
-      <c r="C6" s="26" t="s">
+      <c r="B6" s="14"/>
+      <c r="C6" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="26"/>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
     </row>
     <row r="7" spans="1:7" ht="13.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="25"/>
-      <c r="C7" s="26" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
     </row>
     <row r="9" spans="1:7" ht="14.65" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
     </row>
     <row r="10" spans="1:7" ht="13.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="24" t="s">
+      <c r="A10" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
     </row>
     <row r="11" spans="1:7" ht="13.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="24"/>
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="24"/>
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
     </row>
     <row r="12" spans="1:7" ht="13.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="24"/>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="24"/>
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
     </row>
     <row r="13" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="24"/>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
+      <c r="A13" s="16"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
     </row>
     <row r="15" spans="1:7" ht="14.65" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
     </row>
     <row r="16" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
@@ -1354,7 +1382,7 @@
       </c>
       <c r="E17" s="18"/>
       <c r="F17" s="19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G17" s="19"/>
     </row>
@@ -1369,7 +1397,7 @@
       </c>
       <c r="E18" s="22"/>
       <c r="F18" s="23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G18" s="23"/>
     </row>
@@ -1470,7 +1498,7 @@
         <v>35</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C25" s="17"/>
       <c r="D25" s="18" t="s">
@@ -1478,7 +1506,7 @@
       </c>
       <c r="E25" s="18"/>
       <c r="F25" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G25" s="19"/>
     </row>
@@ -1536,7 +1564,7 @@
       </c>
       <c r="C29" s="17"/>
       <c r="D29" s="18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E29" s="18"/>
       <c r="F29" s="19" t="s">
@@ -1566,7 +1594,7 @@
       </c>
       <c r="C31" s="17"/>
       <c r="D31" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E31" s="18"/>
       <c r="F31" s="19" t="s">
@@ -1575,15 +1603,15 @@
       <c r="G31" s="19"/>
     </row>
     <row r="33" spans="1:7" ht="14.65" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A33" s="14" t="s">
+      <c r="A33" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
     </row>
     <row r="34" spans="1:7" ht="14.65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
@@ -1596,14 +1624,14 @@
         <v>53</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="E34" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="F34" s="16"/>
+      <c r="E34" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="F34" s="28"/>
       <c r="G34" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="160.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -1611,41 +1639,41 @@
         <v>1</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>54</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="E35" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="F35" s="12"/>
+        <v>89</v>
+      </c>
+      <c r="E35" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="F35" s="25"/>
       <c r="G35" s="4" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="146" customHeight="1" x14ac:dyDescent="0.2">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="169" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3">
         <v>2</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C36" s="7" t="s">
         <v>55</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="E36" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="F36" s="11"/>
+        <v>92</v>
+      </c>
+      <c r="E36" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="F36" s="24"/>
       <c r="G36" s="6" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="144.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -1653,20 +1681,20 @@
         <v>3</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>56</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="E37" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="F37" s="12"/>
+        <v>93</v>
+      </c>
+      <c r="E37" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="F37" s="25"/>
       <c r="G37" s="4" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="145.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -1674,18 +1702,18 @@
         <v>4</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C38" s="7" t="s">
         <v>57</v>
       </c>
       <c r="D38" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E38" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="E38" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="F38" s="11"/>
+      <c r="F38" s="24"/>
       <c r="G38" s="6" t="s">
         <v>107</v>
       </c>
@@ -1695,32 +1723,32 @@
         <v>5</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C39" s="5" t="s">
         <v>58</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="E39" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="F39" s="12"/>
+        <v>94</v>
+      </c>
+      <c r="E39" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="F39" s="25"/>
       <c r="G39" s="4" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="14.65" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A41" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
+      <c r="A41" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
     </row>
     <row r="42" spans="1:7" ht="13.4" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
@@ -1732,12 +1760,12 @@
       <c r="C42" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D42" s="15" t="s">
+      <c r="D42" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="E42" s="15"/>
+      <c r="E42" s="27"/>
       <c r="F42" s="1" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="G42" s="1" t="s">
         <v>60</v>
@@ -1753,15 +1781,15 @@
       <c r="C43" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D43" s="12" t="s">
+      <c r="D43" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="E43" s="12"/>
+      <c r="E43" s="25"/>
       <c r="F43" s="4" t="s">
         <v>64</v>
       </c>
       <c r="G43" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="156" customHeight="1" x14ac:dyDescent="0.2">
@@ -1774,10 +1802,10 @@
       <c r="C44" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D44" s="11" t="s">
+      <c r="D44" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="E44" s="11"/>
+      <c r="E44" s="24"/>
       <c r="F44" s="6" t="s">
         <v>68</v>
       </c>
@@ -1795,10 +1823,10 @@
       <c r="C45" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D45" s="12" t="s">
+      <c r="D45" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="E45" s="12"/>
+      <c r="E45" s="25"/>
       <c r="F45" s="4" t="s">
         <v>73</v>
       </c>
@@ -1816,10 +1844,10 @@
       <c r="C46" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D46" s="11" t="s">
+      <c r="D46" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="E46" s="11"/>
+      <c r="E46" s="24"/>
       <c r="F46" s="6" t="s">
         <v>78</v>
       </c>
@@ -1828,78 +1856,18 @@
       </c>
     </row>
     <row r="48" spans="1:7" ht="15" x14ac:dyDescent="0.4">
-      <c r="A48" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="B48" s="13"/>
-      <c r="C48" s="13"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="13"/>
+      <c r="A48" s="29" t="s">
+        <v>111</v>
+      </c>
+      <c r="B48" s="26"/>
+      <c r="C48" s="26"/>
+      <c r="D48" s="26"/>
+      <c r="E48" s="26"/>
+      <c r="F48" s="26"/>
+      <c r="G48" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="76">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A10:G13"/>
-    <mergeCell ref="A15:G15"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="A17:A20"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="A21:A24"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="A25:A28"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="A29:A31"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:G31"/>
     <mergeCell ref="D44:E44"/>
     <mergeCell ref="D45:E45"/>
     <mergeCell ref="D46:E46"/>
@@ -1916,6 +1884,66 @@
     <mergeCell ref="E36:F36"/>
     <mergeCell ref="E37:F37"/>
     <mergeCell ref="B29:C29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="A29:A31"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="A25:A28"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="A10:G13"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="A17:A20"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:G5"/>
   </mergeCells>
   <phoneticPr fontId="12"/>
   <hyperlinks>

</xml_diff>